<commit_message>
docs(modelos): informa o limite de caracteres de cada campo na planilha
Adiciona "(máx. N caracteres)" na descrição dos 35 campos de texto das abas
Produtos, Clientes e Financeiro. Os limites vieram do schema real do SQL Server
(INFORMATION_SCHEMA), não de suposição. Campos numéricos/data mantêm a indicação
de formato (decimal 18,5, flags, AAAA-MM-DD), onde "caracteres" não se aplica.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MaxImporta_Modelos_Importacao.xlsx
+++ b/MaxImporta_Modelos_Importacao.xlsx
@@ -600,35 +600,41 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Descrição do Produto</t>
+          <t>Descrição do Produto
+(máx. 100 caracteres)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Cód. CST2
-(ex: 00,10,20, 60)</t>
+(ex: 00,10,20, 60)
+(máx. 2 caracteres)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Código Interno
-do Produto</t>
+do Produto
+(máx. 50 caracteres)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Unidade
-(ex: PC, KG, CX)</t>
+(ex: PC, KG, CX)
+(máx. 10 caracteres)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Código NCM</t>
+          <t>Código NCM
+(máx. 10 caracteres)</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Aplicação</t>
+          <t>Aplicação
+(texto longo, sem limite)</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -664,7 +670,8 @@
       <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Tipo
-P=Produto  S=Serviço</t>
+P=Produto  S=Serviço
+(máx. 1 caractere)</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
@@ -675,7 +682,8 @@
       </c>
       <c r="O2" s="11" t="inlineStr">
         <is>
-          <t>Cód. CSOSN (ex: 101,102,500)</t>
+          <t>Cód. CSOSN (ex: 101,102,500)
+(máx. 3 caracteres)</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
@@ -704,12 +712,14 @@
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>Localizador</t>
+          <t>Localizador
+(máx. 20 caracteres)</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>Prateleira</t>
+          <t>Prateleira
+(máx. 20 caracteres)</t>
         </is>
       </c>
       <c r="V2" s="3" t="inlineStr">
@@ -721,37 +731,43 @@
       <c r="W2" s="3" t="inlineStr">
         <is>
           <t>Classe do Produto
-(auto-criada)</t>
+(auto-criada)
+(máx. 50 caracteres)</t>
         </is>
       </c>
       <c r="X2" s="3" t="inlineStr">
         <is>
           <t>Código CEST
-(lookup proCEST)</t>
+(lookup proCEST)
+(máx. 10 caracteres)</t>
         </is>
       </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
           <t>Nome do Fabricante
-(auto-criado)</t>
+(auto-criado)
+(máx. 50 caracteres)</t>
         </is>
       </c>
       <c r="Z2" s="3" t="inlineStr">
         <is>
           <t>Grupo do Produto
-(auto-criado)</t>
+(auto-criado)
+(máx. 50 caracteres)</t>
         </is>
       </c>
       <c r="AA2" s="3" t="inlineStr">
         <is>
           <t>SubGrupo do Produto
-(auto-criado)</t>
+(auto-criado)
+(máx. 50 caracteres)</t>
         </is>
       </c>
       <c r="AB2" s="3" t="inlineStr">
         <is>
           <t>Código EAN /
-Código de Barras</t>
+Código de Barras
+(máx. 20 caracteres)</t>
         </is>
       </c>
     </row>
@@ -6948,46 +6964,54 @@
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>CPF / CNPJ
-(sem pontuação)</t>
+(sem pontuação)
+(máx. 20 caracteres)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Razão Social /
-Nome Completo</t>
+Nome Completo
+(máx. 50 caracteres)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Nome Fantasia</t>
+          <t>Nome Fantasia
+(máx. 50 caracteres)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>RG / Insc. Estadual
-(ou ISENTO)</t>
+(ou ISENTO)
+(máx. 20 caracteres)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Endereço de
-Faturamento</t>
+Faturamento
+(máx. 120 caracteres)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Número do
-Endereço</t>
+Endereço
+(máx. 10 caracteres)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Bairro</t>
+          <t>Bairro
+(máx. 70 caracteres)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Cidade</t>
+          <t>Cidade
+(máx. 30 caracteres)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -6999,13 +7023,15 @@
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>UF
-(ex: TO, SP, GO)</t>
+(ex: TO, SP, GO)
+(máx. 2 caracteres)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>CEP
-(8 dígitos, sem hífen)</t>
+(8 dígitos, sem hífen)
+(máx. 9 caracteres)</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -7022,12 +7048,14 @@
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>E-mail</t>
+          <t>E-mail
+(máx. 254 caracteres)</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>Telefone</t>
+          <t>Telefone
+(máx. 20 caracteres)</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
@@ -10972,13 +11000,15 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>CPF / CNPJ
-(lookup cliente)</t>
+(lookup cliente)
+(máx. 20 caracteres)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Nome do Cliente
-no Lançamento</t>
+no Lançamento
+(máx. 50 caracteres)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -11014,23 +11044,27 @@
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Tipo Conta
-R=Receber  P=Pagar</t>
+R=Receber  P=Pagar
+(máx. 1 caractere)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Pago
-C=Quitado  N=Aberto  S=Parcial</t>
+C=Quitado  N=Aberto  S=Parcial
+(máx. 1 caractere)</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Nº do Documento</t>
+          <t>Nº do Documento
+(máx. 30 caracteres)</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Observação</t>
+          <t>Observação
+(máx. 1000 caracteres)</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
@@ -11041,7 +11075,8 @@
       <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Nosso Número
-(boleto)</t>
+(boleto)
+(máx. 30 caracteres)</t>
         </is>
       </c>
     </row>

</xml_diff>